<commit_message>
Refine data cleaning logic and update README based on mentor feedback
</commit_message>
<xml_diff>
--- a/submissions/Project01-MoAminNKC/data/cleaned_dataset.xlsx
+++ b/submissions/Project01-MoAminNKC/data/cleaned_dataset.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q61"/>
+  <dimension ref="A1:R61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -518,6 +518,11 @@
           <t>satisfaction_score</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>returned_items_is_missing</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -530,7 +535,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -586,6 +591,9 @@
       </c>
       <c r="Q2" t="n">
         <v>5</v>
+      </c>
+      <c r="R2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -599,7 +607,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -655,6 +663,9 @@
       </c>
       <c r="Q3" t="n">
         <v>3</v>
+      </c>
+      <c r="R3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -668,7 +679,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -724,6 +735,9 @@
       </c>
       <c r="Q4" t="n">
         <v>1</v>
+      </c>
+      <c r="R4" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -737,7 +751,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -793,6 +807,9 @@
       </c>
       <c r="Q5" t="n">
         <v>4</v>
+      </c>
+      <c r="R5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -806,7 +823,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -862,6 +879,9 @@
       </c>
       <c r="Q6" t="n">
         <v>4</v>
+      </c>
+      <c r="R6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -875,7 +895,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -931,6 +951,9 @@
       </c>
       <c r="Q7" t="n">
         <v>2</v>
+      </c>
+      <c r="R7" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -944,7 +967,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1000,6 +1023,9 @@
       </c>
       <c r="Q8" t="n">
         <v>5</v>
+      </c>
+      <c r="R8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1013,7 +1039,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1068,6 +1094,9 @@
       <c r="Q9" t="n">
         <v>1</v>
       </c>
+      <c r="R9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1080,7 +1109,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -1111,7 +1140,7 @@
         <v>341.63</v>
       </c>
       <c r="K10" t="n">
-        <v>8782.241249999999</v>
+        <v>11615.42</v>
       </c>
       <c r="L10" t="n">
         <v>232</v>
@@ -1136,6 +1165,9 @@
       </c>
       <c r="Q10" t="n">
         <v>2</v>
+      </c>
+      <c r="R10" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1149,7 +1181,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1205,6 +1237,9 @@
       </c>
       <c r="Q11" t="n">
         <v>1</v>
+      </c>
+      <c r="R11" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1275,6 +1310,9 @@
       <c r="Q12" t="n">
         <v>2</v>
       </c>
+      <c r="R12" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1287,7 +1325,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1318,7 +1356,7 @@
         <v>434.5</v>
       </c>
       <c r="K13" t="n">
-        <v>8782.241249999999</v>
+        <v>11731.5</v>
       </c>
       <c r="L13" t="n">
         <v>224</v>
@@ -1343,6 +1381,9 @@
       </c>
       <c r="Q13" t="n">
         <v>2</v>
+      </c>
+      <c r="R13" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1413,6 +1454,9 @@
       <c r="Q14" t="n">
         <v>5</v>
       </c>
+      <c r="R14" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1425,7 +1469,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1481,6 +1525,9 @@
       </c>
       <c r="Q15" t="n">
         <v>4</v>
+      </c>
+      <c r="R15" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -1494,7 +1541,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1549,6 +1596,9 @@
       <c r="Q16" t="n">
         <v>4</v>
       </c>
+      <c r="R16" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1618,6 +1668,9 @@
       <c r="Q17" t="n">
         <v>2</v>
       </c>
+      <c r="R17" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1630,7 +1683,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1686,6 +1739,9 @@
       </c>
       <c r="Q18" t="n">
         <v>4</v>
+      </c>
+      <c r="R18" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1699,7 +1755,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1755,6 +1811,9 @@
       </c>
       <c r="Q19" t="n">
         <v>1</v>
+      </c>
+      <c r="R19" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -1825,6 +1884,9 @@
       <c r="Q20" t="n">
         <v>2</v>
       </c>
+      <c r="R20" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1837,7 +1899,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1893,6 +1955,9 @@
       </c>
       <c r="Q21" t="n">
         <v>5</v>
+      </c>
+      <c r="R21" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -1906,7 +1971,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1962,6 +2027,9 @@
       </c>
       <c r="Q22" t="n">
         <v>1</v>
+      </c>
+      <c r="R22" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -1975,7 +2043,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -2031,6 +2099,9 @@
       </c>
       <c r="Q23" t="n">
         <v>2</v>
+      </c>
+      <c r="R23" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -2044,7 +2115,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -2100,6 +2171,9 @@
       </c>
       <c r="Q24" t="n">
         <v>4</v>
+      </c>
+      <c r="R24" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -2113,7 +2187,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -2168,6 +2242,9 @@
       <c r="Q25" t="n">
         <v>1</v>
       </c>
+      <c r="R25" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2237,6 +2314,9 @@
       <c r="Q26" t="n">
         <v>2</v>
       </c>
+      <c r="R26" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2249,7 +2329,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -2305,6 +2385,9 @@
       </c>
       <c r="Q27" t="n">
         <v>4</v>
+      </c>
+      <c r="R27" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -2318,7 +2401,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -2374,6 +2457,9 @@
       </c>
       <c r="Q28" t="n">
         <v>3</v>
+      </c>
+      <c r="R28" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -2387,7 +2473,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -2443,6 +2529,9 @@
       </c>
       <c r="Q29" t="n">
         <v>5</v>
+      </c>
+      <c r="R29" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -2456,7 +2545,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -2511,6 +2600,9 @@
       <c r="Q30" t="n">
         <v>5</v>
       </c>
+      <c r="R30" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2523,7 +2615,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -2579,6 +2671,9 @@
       </c>
       <c r="Q31" t="n">
         <v>4</v>
+      </c>
+      <c r="R31" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -2592,7 +2687,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -2648,6 +2743,9 @@
       </c>
       <c r="Q32" t="n">
         <v>3</v>
+      </c>
+      <c r="R32" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -2718,6 +2816,9 @@
       <c r="Q33" t="n">
         <v>5</v>
       </c>
+      <c r="R33" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2787,6 +2888,9 @@
       <c r="Q34" t="n">
         <v>5</v>
       </c>
+      <c r="R34" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2799,7 +2903,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -2855,6 +2959,9 @@
       </c>
       <c r="Q35" t="n">
         <v>3</v>
+      </c>
+      <c r="R35" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -2868,7 +2975,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -2924,6 +3031,9 @@
       </c>
       <c r="Q36" t="n">
         <v>3</v>
+      </c>
+      <c r="R36" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -2937,7 +3047,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -2993,6 +3103,9 @@
       </c>
       <c r="Q37" t="n">
         <v>2</v>
+      </c>
+      <c r="R37" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -3006,7 +3119,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -3061,6 +3174,9 @@
       <c r="Q38" t="n">
         <v>2</v>
       </c>
+      <c r="R38" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -3073,7 +3189,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -3129,6 +3245,9 @@
       </c>
       <c r="Q39" t="n">
         <v>4</v>
+      </c>
+      <c r="R39" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -3142,7 +3261,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -3198,6 +3317,9 @@
       </c>
       <c r="Q40" t="n">
         <v>4</v>
+      </c>
+      <c r="R40" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -3211,7 +3333,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -3267,6 +3389,9 @@
       </c>
       <c r="Q41" t="n">
         <v>2</v>
+      </c>
+      <c r="R41" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -3337,6 +3462,9 @@
       <c r="Q42" t="n">
         <v>5</v>
       </c>
+      <c r="R42" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -3349,7 +3477,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -3405,6 +3533,9 @@
       </c>
       <c r="Q43" t="n">
         <v>5</v>
+      </c>
+      <c r="R43" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -3418,7 +3549,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -3474,6 +3605,9 @@
       </c>
       <c r="Q44" t="n">
         <v>4</v>
+      </c>
+      <c r="R44" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -3487,7 +3621,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -3518,7 +3652,7 @@
         <v>434.98</v>
       </c>
       <c r="K45" t="n">
-        <v>8782.241249999999</v>
+        <v>14354.34</v>
       </c>
       <c r="L45" t="n">
         <v>165</v>
@@ -3543,6 +3677,9 @@
       </c>
       <c r="Q45" t="n">
         <v>2</v>
+      </c>
+      <c r="R45" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -3556,7 +3693,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -3612,6 +3749,9 @@
       </c>
       <c r="Q46" t="n">
         <v>1</v>
+      </c>
+      <c r="R46" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -3625,7 +3765,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -3681,6 +3821,9 @@
       </c>
       <c r="Q47" t="n">
         <v>4</v>
+      </c>
+      <c r="R47" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -3694,7 +3837,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -3750,6 +3893,9 @@
       </c>
       <c r="Q48" t="n">
         <v>3</v>
+      </c>
+      <c r="R48" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -3763,7 +3909,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -3819,6 +3965,9 @@
       </c>
       <c r="Q49" t="n">
         <v>2</v>
+      </c>
+      <c r="R49" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -3832,7 +3981,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -3888,6 +4037,9 @@
       </c>
       <c r="Q50" t="n">
         <v>1</v>
+      </c>
+      <c r="R50" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -3901,7 +4053,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -3957,6 +4109,9 @@
       </c>
       <c r="Q51" t="n">
         <v>2</v>
+      </c>
+      <c r="R51" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -3970,7 +4125,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -4026,6 +4181,9 @@
       </c>
       <c r="Q52" t="n">
         <v>5</v>
+      </c>
+      <c r="R52" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -4096,6 +4254,9 @@
       <c r="Q53" t="n">
         <v>3</v>
       </c>
+      <c r="R53" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -4108,7 +4269,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -4164,6 +4325,9 @@
       </c>
       <c r="Q54" t="n">
         <v>1</v>
+      </c>
+      <c r="R54" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -4177,7 +4341,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -4233,6 +4397,9 @@
       </c>
       <c r="Q55" t="n">
         <v>1</v>
+      </c>
+      <c r="R55" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -4246,7 +4413,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -4302,6 +4469,9 @@
       </c>
       <c r="Q56" t="n">
         <v>1</v>
+      </c>
+      <c r="R56" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -4315,7 +4485,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -4370,6 +4540,9 @@
       <c r="Q57" t="n">
         <v>2</v>
       </c>
+      <c r="R57" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -4382,7 +4555,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -4413,7 +4586,7 @@
         <v>436.54</v>
       </c>
       <c r="K58" t="n">
-        <v>8782.241249999999</v>
+        <v>13532.74</v>
       </c>
       <c r="L58" t="n">
         <v>82</v>
@@ -4438,6 +4611,9 @@
       </c>
       <c r="Q58" t="n">
         <v>4</v>
+      </c>
+      <c r="R58" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -4451,7 +4627,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -4507,6 +4683,9 @@
       </c>
       <c r="Q59" t="n">
         <v>2</v>
+      </c>
+      <c r="R59" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -4520,7 +4699,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -4551,7 +4730,7 @@
         <v>287.05</v>
       </c>
       <c r="K60" t="n">
-        <v>8782.241249999999</v>
+        <v>8898.549999999999</v>
       </c>
       <c r="L60" t="n">
         <v>224</v>
@@ -4576,6 +4755,9 @@
       </c>
       <c r="Q60" t="n">
         <v>5</v>
+      </c>
+      <c r="R60" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -4589,7 +4771,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -4645,6 +4827,9 @@
       </c>
       <c r="Q61" t="n">
         <v>3</v>
+      </c>
+      <c r="R61" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>